<commit_message>
update cfd data and aerodynamic modeling script
</commit_message>
<xml_diff>
--- a/aerodynamic-modeling/linear_regression_cfd/CFD_Data_Collection.xlsx
+++ b/aerodynamic-modeling/linear_regression_cfd/CFD_Data_Collection.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Beta=180" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="47">
   <si>
     <t xml:space="preserve">Beta=180 deg</t>
   </si>
@@ -35,19 +35,119 @@
     <t xml:space="preserve"> m/s</t>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=150 degree</t>
+    <t xml:space="preserve">Overall Alpha Angle=150 degree</t>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=120 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=120 degree</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=90 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=90 degree</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=60 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=60 degree</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=30 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=30 degree</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">link name</t>
@@ -68,19 +168,13 @@
     <t xml:space="preserve">Drag</t>
   </si>
   <si>
-    <t xml:space="preserve">Lift</t>
+    <t xml:space="preserve">Normal</t>
   </si>
   <si>
     <t xml:space="preserve">C_D</t>
   </si>
   <si>
-    <t xml:space="preserve">C_L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Drag </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lift </t>
+    <t xml:space="preserve">C_N</t>
   </si>
   <si>
     <t xml:space="preserve">head</t>
@@ -128,16 +222,116 @@
     <t xml:space="preserve">Beta=270 deg</t>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=180 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=180 degree</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=160 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=160 degree</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=45 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=45 degree</t>
+    </r>
   </si>
   <si>
-    <t xml:space="preserve">Overall Angle of Attack=15 degree</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Overall </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Alpha Angle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=15 degree</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Alpha=90 deg</t>
@@ -324,7 +518,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -421,10 +615,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -503,7 +693,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC35"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="7.22"/>
@@ -615,66 +805,66 @@
         <v>12</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="O2" s="19" t="s">
         <v>12</v>
       </c>
       <c r="P2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="Q2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="R2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="T2" s="19" t="s">
         <v>12</v>
       </c>
       <c r="U2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="V2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="W2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="X2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="Y2" s="19" t="s">
         <v>12</v>
       </c>
       <c r="Z2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AA2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="AB2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AC2" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>0.0429</v>
@@ -774,7 +964,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>0.153</v>
@@ -874,7 +1064,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>0.0484</v>
@@ -974,7 +1164,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>0.0136</v>
@@ -1074,7 +1264,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>0.0136</v>
@@ -1174,7 +1364,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>0.0433</v>
@@ -1274,7 +1464,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>0.0433</v>
@@ -1374,7 +1564,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>0.0247</v>
@@ -1474,7 +1664,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>0.0247</v>
@@ -1574,7 +1764,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>0.026</v>
@@ -1674,7 +1864,7 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>0.026</v>
@@ -1774,7 +1964,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>0.0052</v>
@@ -1874,7 +2064,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>0.0052</v>
@@ -1974,7 +2164,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>7.5</v>
@@ -2237,7 +2427,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC16"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.57"/>
@@ -2260,7 +2450,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="29.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>1</v>
@@ -2270,14 +2460,14 @@
         <v>2</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
       <c r="J1" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
@@ -2291,14 +2481,14 @@
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
       <c r="T1" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="U1" s="10"/>
       <c r="V1" s="10"/>
       <c r="W1" s="10"/>
       <c r="X1" s="10"/>
       <c r="Y1" s="10" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Z1" s="10"/>
       <c r="AA1" s="10"/>
@@ -2337,66 +2527,66 @@
         <v>12</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="O2" s="19" t="s">
         <v>12</v>
       </c>
       <c r="P2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="Q2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="R2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="T2" s="19" t="s">
         <v>12</v>
       </c>
       <c r="U2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="V2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="W2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="X2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="Y2" s="19" t="s">
         <v>12</v>
       </c>
       <c r="Z2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AA2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="AB2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AC2" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>0.0429</v>
@@ -2496,7 +2686,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>0.153</v>
@@ -2596,7 +2786,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>0.0484</v>
@@ -2696,7 +2886,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>0.0136</v>
@@ -2796,7 +2986,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>0.0136</v>
@@ -2896,7 +3086,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>0.0433</v>
@@ -2996,7 +3186,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>0.0433</v>
@@ -3096,7 +3286,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>0.0247</v>
@@ -3196,7 +3386,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>0.0247</v>
@@ -3296,7 +3486,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>0.026</v>
@@ -3396,7 +3586,7 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>0.026</v>
@@ -3496,7 +3686,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>0.0052</v>
@@ -3596,7 +3786,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>0.0052</v>
@@ -3696,7 +3886,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>7.5</v>
@@ -3821,7 +4011,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC25"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.57"/>
@@ -3844,7 +4034,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="29.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>1</v>
@@ -3854,35 +4044,35 @@
         <v>2</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
       <c r="J1" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
       <c r="M1" s="10"/>
       <c r="N1" s="10"/>
       <c r="O1" s="10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="P1" s="10"/>
       <c r="Q1" s="10"/>
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
       <c r="T1" s="10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="U1" s="10"/>
       <c r="V1" s="10"/>
       <c r="W1" s="10"/>
       <c r="X1" s="10"/>
       <c r="Y1" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z1" s="10"/>
       <c r="AA1" s="10"/>
@@ -3903,84 +4093,84 @@
         <v>11</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="J2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="O2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="P2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="Q2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="R2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="T2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="U2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="V2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="W2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="X2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="Y2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Z2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AA2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="AB2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AC2" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>0.0429</v>
@@ -4067,7 +4257,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>0.153</v>
@@ -4154,7 +4344,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>0.0484</v>
@@ -4241,7 +4431,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>0.0136</v>
@@ -4328,7 +4518,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>0.0136</v>
@@ -4415,7 +4605,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>0.0433</v>
@@ -4502,7 +4692,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>0.0433</v>
@@ -4589,7 +4779,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>0.0247</v>
@@ -4676,7 +4866,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>0.0247</v>
@@ -4763,7 +4953,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>0.026</v>
@@ -4850,7 +5040,7 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>0.026</v>
@@ -4937,7 +5127,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>0.0052</v>
@@ -5024,7 +5214,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>0.0052</v>
@@ -5111,7 +5301,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>7.5</v>
@@ -5246,7 +5436,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC17"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.57"/>
@@ -5269,7 +5459,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="29.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>1</v>
@@ -5279,35 +5469,35 @@
         <v>2</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
       <c r="J1" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
       <c r="M1" s="10"/>
       <c r="N1" s="10"/>
       <c r="O1" s="10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="P1" s="10"/>
       <c r="Q1" s="10"/>
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
-      <c r="T1" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="U1" s="24"/>
-      <c r="V1" s="24"/>
-      <c r="W1" s="24"/>
-      <c r="X1" s="24"/>
+      <c r="T1" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
       <c r="Y1" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z1" s="10"/>
       <c r="AA1" s="10"/>
@@ -5328,84 +5518,84 @@
         <v>11</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="J2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="O2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="P2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="Q2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="R2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="T2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="U2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="V2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="W2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="X2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="Y2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="Z2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AA2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="AB2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AC2" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>0.0429</v>
@@ -5492,7 +5682,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>0.153</v>
@@ -5579,7 +5769,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>0.0484</v>
@@ -5666,7 +5856,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>0.0136</v>
@@ -5753,7 +5943,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>0.0136</v>
@@ -5840,7 +6030,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>0.0433</v>
@@ -5927,7 +6117,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>0.0433</v>
@@ -6014,7 +6204,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>0.0247</v>
@@ -6101,7 +6291,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>0.0247</v>
@@ -6188,7 +6378,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>0.026</v>
@@ -6275,7 +6465,7 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>0.026</v>
@@ -6362,7 +6552,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>0.0052</v>
@@ -6449,7 +6639,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>0.0052</v>
@@ -6536,7 +6726,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>7.5</v>
@@ -6668,7 +6858,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC17"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.57"/>
@@ -6691,7 +6881,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="29.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>1</v>
@@ -6701,35 +6891,35 @@
         <v>2</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
       <c r="I1" s="9"/>
       <c r="J1" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K1" s="10"/>
       <c r="L1" s="10"/>
       <c r="M1" s="10"/>
       <c r="N1" s="10"/>
       <c r="O1" s="10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="P1" s="10"/>
       <c r="Q1" s="10"/>
       <c r="R1" s="10"/>
       <c r="S1" s="10"/>
       <c r="T1" s="10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="U1" s="10"/>
       <c r="V1" s="10"/>
       <c r="W1" s="10"/>
       <c r="X1" s="10"/>
       <c r="Y1" s="10" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Z1" s="10"/>
       <c r="AA1" s="10"/>
@@ -6750,84 +6940,84 @@
         <v>11</v>
       </c>
       <c r="E2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="H2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="J2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="O2" s="19" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="P2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="Q2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="R2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="S2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="T2" s="19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="U2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="V2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="W2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="X2" s="4" t="s">
         <v>16</v>
       </c>
       <c r="Y2" s="19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="Z2" s="16" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AA2" s="17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="AB2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="AC2" s="3" t="s">
+      <c r="AC2" s="4" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>0.0429</v>
@@ -6914,7 +7104,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>0.153</v>
@@ -7001,7 +7191,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>0.0484</v>
@@ -7088,7 +7278,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>0.0136</v>
@@ -7175,7 +7365,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>0.0136</v>
@@ -7262,7 +7452,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>0.0433</v>
@@ -7349,7 +7539,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>0.0433</v>
@@ -7436,7 +7626,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>0.0247</v>
@@ -7523,7 +7713,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>0.0247</v>
@@ -7610,7 +7800,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>0.026</v>
@@ -7697,7 +7887,7 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>0.026</v>
@@ -7784,7 +7974,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>0.0052</v>
@@ -7871,7 +8061,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>0.0052</v>
@@ -7958,7 +8148,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>7.5</v>

</xml_diff>